<commit_message>
Etapa 13: respaldo programado con retención y riesgo residual sin altos
</commit_message>
<xml_diff>
--- a/docs/analisis-de-riesgos-cms.xlsx
+++ b/docs/analisis-de-riesgos-cms.xlsx
@@ -1604,13 +1604,13 @@
     <t xml:space="preserve">Diseñado</t>
   </si>
   <si>
-    <t xml:space="preserve">Volumen persistente en Docker. Diseño cloud: respaldos de 14 días y protección contra borrado. Residual: sin respaldo automatizado en el entorno local.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 8A (persistencia); Terraform.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brecha abierta: el entorno local no tiene respaldo automático. Diseño cloud con 14 días de respaldo. Se baja a 1 al probar un respaldo y su restauración.</t>
+    <t xml:space="preserve">Volumen persistente en Docker y respaldo diario con mongodump (script backup/respaldo.ps1, retención de 14 días) con prueba de restauración. Diseño cloud: respaldos de 14 días y protección contra borrado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 8A (persistencia); docs/evidencias/respaldo-restauracion.txt (116 documentos restaurados, 0 fallos); Terraform.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Respaldo diario programado con retención de 14 días y restauración verificada en bases temporales. Residual: el respaldo está en el mismo equipo (convendría una copia externa) y depende de que la PC esté encendida.</t>
   </si>
   <si>
     <t xml:space="preserve">Humano</t>
@@ -1979,7 +1979,7 @@
     <t xml:space="preserve">T-12, T-13, T-23, T-25</t>
   </si>
   <si>
-    <t xml:space="preserve">La llave de cifrado está en el mismo servidor que los datos. No hay respaldo automatizado en el entorno local. Certificado autofirmado local.</t>
+    <t xml:space="preserve">La llave de cifrado está en el mismo servidor que los datos. El respaldo es manual (script con restauración probada) y falta programarlo. Certificado autofirmado local.</t>
   </si>
   <si>
     <t xml:space="preserve">Etapas 7B, 8B y 9; Gitleaks sin fugas.</t>
@@ -2318,7 +2318,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2385,14 +2385,6 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2829,7 +2821,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
@@ -6480,8 +6472,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8049,18 +8041,18 @@
         <v>524</v>
       </c>
       <c r="K29" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L29" s="16" t="n">
         <v>5</v>
       </c>
       <c r="M29" s="12" t="n">
         <f aca="false">IF(OR(K29="",L29=""),"",K29*L29)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N29" s="12" t="str">
         <f aca="false">IF(M29="","",IF(M29&gt;=Escalas!$B$13,"Crítico",IF(M29&gt;=Escalas!$B$14,"Alto",IF(M29&gt;=Escalas!$B$15,"Medio","Bajo"))))</f>
-        <v>Alto</v>
+        <v>Medio</v>
       </c>
       <c r="O29" s="16" t="s">
         <v>442</v>
@@ -8069,7 +8061,7 @@
         <v>525</v>
       </c>
       <c r="Q29" s="16" t="s">
-        <v>493</v>
+        <v>444</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8359,28 +8351,28 @@
   <dimension ref="A1:P25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>540</v>
       </c>
     </row>
@@ -8434,7 +8426,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
         <v>552</v>
       </c>
@@ -8486,7 +8478,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
         <v>559</v>
       </c>
@@ -8538,7 +8530,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
         <v>563</v>
       </c>
@@ -8578,7 +8570,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
         <v>569</v>
       </c>
@@ -8630,7 +8622,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
         <v>574</v>
       </c>
@@ -8682,7 +8674,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
         <v>579</v>
       </c>
@@ -8734,7 +8726,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
         <v>584</v>
       </c>
@@ -8786,7 +8778,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
         <v>589</v>
       </c>
@@ -8836,7 +8828,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
         <v>593</v>
       </c>
@@ -8888,7 +8880,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
         <v>598</v>
       </c>
@@ -8930,7 +8922,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>603</v>
       </c>
@@ -8982,7 +8974,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
         <v>608</v>
       </c>
@@ -9034,7 +9026,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
         <v>613</v>
       </c>
@@ -9086,7 +9078,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
         <v>618</v>
       </c>
@@ -9128,7 +9120,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
         <v>622</v>
       </c>
@@ -9139,7 +9131,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
         <v>556</v>
       </c>
@@ -9152,7 +9144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="5" t="s">
         <v>567</v>
       </c>
@@ -9165,7 +9157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="5" t="s">
         <v>557</v>
       </c>
@@ -9178,7 +9170,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="5" t="s">
         <v>478</v>
       </c>
@@ -9191,7 +9183,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="11" t="s">
         <v>260</v>
       </c>
@@ -9256,7 +9248,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="14" t="s">
         <v>628</v>
       </c>
@@ -9275,7 +9267,7 @@
       <c r="G5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="18" t="s">
         <v>629</v>
       </c>
     </row>
@@ -9286,23 +9278,23 @@
       <c r="B6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B6,Matriz!$F$5:$F$33,C$5)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B6,Matriz!$F$5:$F$33,D$5)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B6,Matriz!$F$5:$F$33,E$5)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="21" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B6,Matriz!$F$5:$F$33,F$5)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="21" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B6,Matriz!$F$5:$F$33,G$5)</f>
         <v>0</v>
       </c>
@@ -9314,23 +9306,23 @@
       <c r="B7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B7,Matriz!$F$5:$F$33,C$5)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B7,Matriz!$F$5:$F$33,D$5)</f>
         <v>2</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B7,Matriz!$F$5:$F$33,E$5)</f>
         <v>2</v>
       </c>
-      <c r="F7" s="22" t="n">
+      <c r="F7" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B7,Matriz!$F$5:$F$33,F$5)</f>
         <v>2</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="21" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B7,Matriz!$F$5:$F$33,G$5)</f>
         <v>2</v>
       </c>
@@ -9342,23 +9334,23 @@
       <c r="B8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B8,Matriz!$F$5:$F$33,C$5)</f>
         <v>1</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B8,Matriz!$F$5:$F$33,D$5)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B8,Matriz!$F$5:$F$33,E$5)</f>
         <v>4</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B8,Matriz!$F$5:$F$33,F$5)</f>
         <v>6</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B8,Matriz!$F$5:$F$33,G$5)</f>
         <v>3</v>
       </c>
@@ -9370,23 +9362,23 @@
       <c r="B9" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B9,Matriz!$F$5:$F$33,C$5)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B9,Matriz!$F$5:$F$33,D$5)</f>
         <v>1</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B9,Matriz!$F$5:$F$33,E$5)</f>
         <v>1</v>
       </c>
-      <c r="F9" s="21" t="n">
+      <c r="F9" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B9,Matriz!$F$5:$F$33,F$5)</f>
         <v>1</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B9,Matriz!$F$5:$F$33,G$5)</f>
         <v>4</v>
       </c>
@@ -9398,23 +9390,23 @@
       <c r="B10" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B10,Matriz!$F$5:$F$33,C$5)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B10,Matriz!$F$5:$F$33,D$5)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B10,Matriz!$F$5:$F$33,E$5)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B10,Matriz!$F$5:$F$33,F$5)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$E$5:$E$33,$B10,Matriz!$F$5:$F$33,G$5)</f>
         <v>0</v>
       </c>
@@ -9425,7 +9417,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19"/>
+      <c r="A15" s="17"/>
       <c r="B15" s="14" t="s">
         <v>628</v>
       </c>
@@ -9444,7 +9436,7 @@
       <c r="G15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="18" t="s">
         <v>629</v>
       </c>
     </row>
@@ -9455,23 +9447,23 @@
       <c r="B16" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B16,Matriz!$L$5:$L$33,C$15)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="D16" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B16,Matriz!$L$5:$L$33,D$15)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B16,Matriz!$L$5:$L$33,E$15)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="23" t="n">
+      <c r="F16" s="21" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B16,Matriz!$L$5:$L$33,F$15)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="23" t="n">
+      <c r="G16" s="21" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B16,Matriz!$L$5:$L$33,G$15)</f>
         <v>0</v>
       </c>
@@ -9483,23 +9475,23 @@
       <c r="B17" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B17,Matriz!$L$5:$L$33,C$15)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B17,Matriz!$L$5:$L$33,D$15)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B17,Matriz!$L$5:$L$33,E$15)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="22" t="n">
+      <c r="F17" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B17,Matriz!$L$5:$L$33,F$15)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="23" t="n">
+      <c r="G17" s="21" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B17,Matriz!$L$5:$L$33,G$15)</f>
         <v>0</v>
       </c>
@@ -9511,23 +9503,23 @@
       <c r="B18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B18,Matriz!$L$5:$L$33,C$15)</f>
         <v>1</v>
       </c>
-      <c r="D18" s="21" t="n">
+      <c r="D18" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B18,Matriz!$L$5:$L$33,D$15)</f>
         <v>1</v>
       </c>
-      <c r="E18" s="21" t="n">
+      <c r="E18" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B18,Matriz!$L$5:$L$33,E$15)</f>
         <v>1</v>
       </c>
-      <c r="F18" s="22" t="n">
+      <c r="F18" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B18,Matriz!$L$5:$L$33,F$15)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="22" t="n">
+      <c r="G18" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B18,Matriz!$L$5:$L$33,G$15)</f>
         <v>0</v>
       </c>
@@ -9539,25 +9531,25 @@
       <c r="B19" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B19,Matriz!$L$5:$L$33,C$15)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B19,Matriz!$L$5:$L$33,D$15)</f>
         <v>2</v>
       </c>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B19,Matriz!$L$5:$L$33,E$15)</f>
         <v>5</v>
       </c>
-      <c r="F19" s="21" t="n">
+      <c r="F19" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B19,Matriz!$L$5:$L$33,F$15)</f>
         <v>3</v>
       </c>
-      <c r="G19" s="22" t="n">
+      <c r="G19" s="20" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B19,Matriz!$L$5:$L$33,G$15)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9567,25 +9559,25 @@
       <c r="B20" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B20,Matriz!$L$5:$L$33,C$15)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B20,Matriz!$L$5:$L$33,D$15)</f>
         <v>1</v>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="E20" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B20,Matriz!$L$5:$L$33,E$15)</f>
         <v>5</v>
       </c>
-      <c r="F20" s="24" t="n">
+      <c r="F20" s="22" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B20,Matriz!$L$5:$L$33,F$15)</f>
         <v>4</v>
       </c>
-      <c r="G20" s="21" t="n">
+      <c r="G20" s="19" t="n">
         <f aca="false">COUNTIFS(Matriz!$K$5:$K$33,$B20,Matriz!$L$5:$L$33,G$15)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9605,7 +9597,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="23" t="s">
         <v>636</v>
       </c>
       <c r="B26" s="12" t="n">
@@ -9618,7 +9610,7 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="24" t="s">
         <v>418</v>
       </c>
       <c r="B27" s="12" t="n">
@@ -9627,11 +9619,11 @@
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">COUNTIF(Matriz!$N$5:$N$33,A27)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="25" t="s">
         <v>419</v>
       </c>
       <c r="B28" s="12" t="n">
@@ -9640,11 +9632,11 @@
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">COUNTIF(Matriz!$N$5:$N$33,A28)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="26" t="s">
         <v>420</v>
       </c>
       <c r="B29" s="12" t="n">

</xml_diff>